<commit_message>
Fix price consistency and add end-to-end project summary
Align leftover 470 TL/m² artifacts to canonical kırık×450, refresh
okul/kalıp payı and hakediş tables, update phone index, add PROJE_OZET.

Co-authored-by: barsokrr <barsokrr@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/metraj/Kalip_Fiyat_Kiyaslama_2026.xlsx
+++ b/metraj/Kalip_Fiyat_Kiyaslama_2026.xlsx
@@ -1241,7 +1241,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -1255,6 +1255,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
@@ -1275,7 +1276,7 @@
       </c>
       <c r="B4" s="12" t="inlineStr">
         <is>
-          <t>470 TL/m²</t>
+          <t>450 TL/m² (güncel); eski 470 referans</t>
         </is>
       </c>
     </row>
@@ -1342,12 +1343,12 @@
     <row r="10">
       <c r="A10" s="12" t="inlineStr">
         <is>
-          <t>Kırık 470 değerlendirme</t>
+          <t>Kırık 450 değerlendirme</t>
         </is>
       </c>
       <c r="B10" s="12" t="inlineStr">
         <is>
-          <t>Gerçekçi (işçilik)</t>
+          <t>Gerçekçi (işçilik) — okul bandı içinde</t>
         </is>
       </c>
     </row>
@@ -1366,12 +1367,12 @@
     <row r="12">
       <c r="A12" s="12" t="inlineStr">
         <is>
-          <t>Kırık metraj × 470</t>
+          <t>Kırık metraj × 450</t>
         </is>
       </c>
       <c r="B12" s="12" t="inlineStr">
         <is>
-          <t>5533498 TL</t>
+          <t>5298030.0 TL</t>
         </is>
       </c>
     </row>
@@ -1399,6 +1400,12 @@
         </is>
       </c>
     </row>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>